<commit_message>
updating processor moodule to include CDM views
</commit_message>
<xml_diff>
--- a/cfihos_src/cdm_export.xlsx
+++ b/cfihos_src/cdm_export.xlsx
@@ -2575,7 +2575,7 @@
     <col min="16" max="16" style="10" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18" hidden="1">
       <c r="A1" s="4" t="s">
         <v>203</v>
       </c>
@@ -2595,7 +2595,7 @@
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18" hidden="1">
       <c r="A2" s="5" t="s">
         <v>104</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18" hidden="1">
       <c r="A3" s="6" t="s">
         <v>82</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>218</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18" hidden="1">
       <c r="A4" s="6" t="s">
         <v>82</v>
       </c>
@@ -2729,7 +2729,7 @@
         <v>223</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18" hidden="1">
       <c r="A5" s="6" t="s">
         <v>82</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>228</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18" hidden="1">
       <c r="A6" s="6" t="s">
         <v>82</v>
       </c>
@@ -2811,7 +2811,7 @@
         <v>233</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18" hidden="1">
       <c r="A7" s="6" t="s">
         <v>82</v>
       </c>
@@ -2853,7 +2853,7 @@
         <v>236</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18" hidden="1">
       <c r="A8" s="6" t="s">
         <v>82</v>
       </c>
@@ -2895,7 +2895,7 @@
         <v>239</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18" hidden="1">
       <c r="A9" s="6" t="s">
         <v>82</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>244</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18" hidden="1">
       <c r="A10" s="6" t="s">
         <v>82</v>
       </c>
@@ -2963,7 +2963,7 @@
         <v>249</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18" hidden="1">
       <c r="A11" s="6" t="s">
         <v>82</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>253</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18" hidden="1">
       <c r="A12" s="6" t="s">
         <v>82</v>
       </c>
@@ -3031,7 +3031,7 @@
         <v>257</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18" hidden="1">
       <c r="A13" s="6" t="s">
         <v>82</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>260</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18" hidden="1">
       <c r="A14" s="8" t="s">
         <v>85</v>
       </c>
@@ -3105,7 +3105,7 @@
         <v>263</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18" hidden="1">
       <c r="A15" s="8" t="s">
         <v>85</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>266</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18" hidden="1">
       <c r="A16" s="8" t="s">
         <v>85</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>269</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18" hidden="1">
       <c r="A17" s="8" t="s">
         <v>85</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>272</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18" hidden="1">
       <c r="A18" s="6" t="s">
         <v>115</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>275</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18" hidden="1">
       <c r="A19" s="6" t="s">
         <v>115</v>
       </c>
@@ -3305,7 +3305,7 @@
         <v>278</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18" hidden="1">
       <c r="A20" s="6" t="s">
         <v>115</v>
       </c>
@@ -3383,7 +3383,7 @@
         <v>284</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18" hidden="1">
       <c r="A22" s="6" t="s">
         <v>115</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>288</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18" hidden="1">
       <c r="A23" s="6" t="s">
         <v>115</v>
       </c>
@@ -3459,7 +3459,7 @@
         <v>291</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18" hidden="1">
       <c r="A24" s="6" t="s">
         <v>115</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>294</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18" hidden="1">
       <c r="A25" s="8" t="s">
         <v>118</v>
       </c>
@@ -3537,7 +3537,7 @@
         <v>296</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18" hidden="1">
       <c r="A26" s="8" t="s">
         <v>118</v>
       </c>
@@ -3575,7 +3575,7 @@
         <v>299</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18" hidden="1">
       <c r="A27" s="6" t="s">
         <v>59</v>
       </c>
@@ -3613,7 +3613,7 @@
         <v>302</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18" hidden="1">
       <c r="A28" s="6" t="s">
         <v>59</v>
       </c>
@@ -3651,7 +3651,7 @@
         <v>306</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18" hidden="1">
       <c r="A29" s="8" t="s">
         <v>124</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>309</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18" hidden="1">
       <c r="A30" s="8" t="s">
         <v>124</v>
       </c>
@@ -3727,7 +3727,7 @@
         <v>312</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18" hidden="1">
       <c r="A31" s="8" t="s">
         <v>124</v>
       </c>
@@ -3765,7 +3765,7 @@
         <v>315</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18" hidden="1">
       <c r="A32" s="8" t="s">
         <v>124</v>
       </c>
@@ -3803,7 +3803,7 @@
         <v>318</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18" hidden="1">
       <c r="A33" s="8" t="s">
         <v>124</v>
       </c>
@@ -3841,7 +3841,7 @@
         <v>321</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18" hidden="1">
       <c r="A34" s="8" t="s">
         <v>124</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>324</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18" hidden="1">
       <c r="A35" s="8" t="s">
         <v>124</v>
       </c>
@@ -3917,7 +3917,7 @@
         <v>327</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18" hidden="1">
       <c r="A36" s="8" t="s">
         <v>124</v>
       </c>
@@ -3955,7 +3955,7 @@
         <v>330</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18" hidden="1">
       <c r="A37" s="8" t="s">
         <v>124</v>
       </c>
@@ -3993,7 +3993,7 @@
         <v>333</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18" hidden="1">
       <c r="A38" s="6" t="s">
         <v>90</v>
       </c>
@@ -4035,7 +4035,7 @@
         <v>337</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18" hidden="1">
       <c r="A39" s="6" t="s">
         <v>90</v>
       </c>
@@ -4077,7 +4077,7 @@
         <v>339</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18" hidden="1">
       <c r="A40" s="6" t="s">
         <v>90</v>
       </c>
@@ -4119,7 +4119,7 @@
         <v>341</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18" hidden="1">
       <c r="A41" s="8" t="s">
         <v>130</v>
       </c>
@@ -4159,7 +4159,7 @@
         <v>342</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18" hidden="1">
       <c r="A42" s="8" t="s">
         <v>130</v>
       </c>
@@ -4199,7 +4199,7 @@
         <v>344</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18" hidden="1">
       <c r="A43" s="8" t="s">
         <v>130</v>
       </c>
@@ -4277,7 +4277,7 @@
         <v>349</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18" hidden="1">
       <c r="A45" s="8" t="s">
         <v>130</v>
       </c>
@@ -4315,7 +4315,7 @@
         <v>352</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18" hidden="1">
       <c r="A46" s="8" t="s">
         <v>130</v>
       </c>
@@ -4353,7 +4353,7 @@
         <v>355</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18" hidden="1">
       <c r="A47" s="6" t="s">
         <v>98</v>
       </c>
@@ -4395,7 +4395,7 @@
         <v>358</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18" hidden="1">
       <c r="A48" s="6" t="s">
         <v>98</v>
       </c>
@@ -4437,7 +4437,7 @@
         <v>362</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18" hidden="1">
       <c r="A49" s="6" t="s">
         <v>98</v>
       </c>
@@ -4479,7 +4479,7 @@
         <v>366</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18" hidden="1">
       <c r="A50" s="6" t="s">
         <v>98</v>
       </c>
@@ -4521,7 +4521,7 @@
         <v>369</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18" hidden="1">
       <c r="A51" s="6" t="s">
         <v>98</v>
       </c>
@@ -4563,7 +4563,7 @@
         <v>371</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18" hidden="1">
       <c r="A52" s="6" t="s">
         <v>98</v>
       </c>
@@ -4597,7 +4597,7 @@
         <v>374</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18" hidden="1">
       <c r="A53" s="6" t="s">
         <v>98</v>
       </c>
@@ -4631,7 +4631,7 @@
         <v>376</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18" hidden="1">
       <c r="A54" s="8" t="s">
         <v>93</v>
       </c>
@@ -4669,7 +4669,7 @@
         <v>379</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18" hidden="1">
       <c r="A55" s="8" t="s">
         <v>93</v>
       </c>
@@ -4707,7 +4707,7 @@
         <v>382</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18" hidden="1">
       <c r="A56" s="8" t="s">
         <v>93</v>
       </c>
@@ -4745,7 +4745,7 @@
         <v>385</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18" hidden="1">
       <c r="A57" s="8" t="s">
         <v>93</v>
       </c>
@@ -4783,7 +4783,7 @@
         <v>388</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18" hidden="1">
       <c r="A58" s="6" t="s">
         <v>55</v>
       </c>
@@ -4825,7 +4825,7 @@
         <v>393</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18" hidden="1">
       <c r="A59" s="6" t="s">
         <v>55</v>
       </c>
@@ -4867,7 +4867,7 @@
         <v>397</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18" hidden="1">
       <c r="A60" s="8" t="s">
         <v>71</v>
       </c>
@@ -4909,7 +4909,7 @@
         <v>399</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18" hidden="1">
       <c r="A61" s="8" t="s">
         <v>71</v>
       </c>
@@ -4949,7 +4949,7 @@
         <v>403</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18" hidden="1">
       <c r="A62" s="8" t="s">
         <v>71</v>
       </c>
@@ -4991,7 +4991,7 @@
         <v>405</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18" hidden="1">
       <c r="A63" s="8" t="s">
         <v>71</v>
       </c>
@@ -5031,7 +5031,7 @@
         <v>409</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18" hidden="1">
       <c r="A64" s="6" t="s">
         <v>143</v>
       </c>
@@ -5071,7 +5071,7 @@
         <v>412</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18" hidden="1">
       <c r="A65" s="6" t="s">
         <v>143</v>
       </c>
@@ -5109,7 +5109,7 @@
         <v>415</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18" hidden="1">
       <c r="A66" s="8" t="s">
         <v>120</v>
       </c>
@@ -5145,7 +5145,7 @@
         <v>417</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18" hidden="1">
       <c r="A67" s="8" t="s">
         <v>120</v>
       </c>
@@ -5181,7 +5181,7 @@
         <v>419</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18" hidden="1">
       <c r="A68" s="8" t="s">
         <v>120</v>
       </c>
@@ -5217,7 +5217,7 @@
         <v>421</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18" hidden="1">
       <c r="A69" s="8" t="s">
         <v>120</v>
       </c>
@@ -5255,7 +5255,7 @@
         <v>422</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18" hidden="1">
       <c r="A70" s="6" t="s">
         <v>148</v>
       </c>
@@ -5295,7 +5295,7 @@
         <v>425</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18" hidden="1">
       <c r="A71" s="6" t="s">
         <v>148</v>
       </c>
@@ -5335,7 +5335,7 @@
         <v>428</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18" hidden="1">
       <c r="A72" s="6" t="s">
         <v>148</v>
       </c>
@@ -5375,7 +5375,7 @@
         <v>431</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18" hidden="1">
       <c r="A73" s="6" t="s">
         <v>148</v>
       </c>
@@ -5415,7 +5415,7 @@
         <v>434</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18" hidden="1">
       <c r="A74" s="6" t="s">
         <v>148</v>
       </c>
@@ -5455,7 +5455,7 @@
         <v>437</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18" hidden="1">
       <c r="A75" s="6" t="s">
         <v>148</v>
       </c>
@@ -5527,7 +5527,7 @@
         <v>443</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18" hidden="1">
       <c r="A77" s="6" t="s">
         <v>88</v>
       </c>
@@ -5569,7 +5569,7 @@
         <v>447</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18" hidden="1">
       <c r="A78" s="6" t="s">
         <v>88</v>
       </c>
@@ -5609,7 +5609,7 @@
         <v>451</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18" hidden="1">
       <c r="A79" s="6" t="s">
         <v>88</v>
       </c>
@@ -5649,7 +5649,7 @@
         <v>455</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18" hidden="1">
       <c r="A80" s="6" t="s">
         <v>88</v>
       </c>
@@ -5691,7 +5691,7 @@
         <v>459</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18" hidden="1">
       <c r="A81" s="6" t="s">
         <v>88</v>
       </c>
@@ -5733,7 +5733,7 @@
         <v>461</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18" hidden="1">
       <c r="A82" s="6" t="s">
         <v>88</v>
       </c>
@@ -5775,7 +5775,7 @@
         <v>463</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18" hidden="1">
       <c r="A83" s="6" t="s">
         <v>88</v>
       </c>
@@ -5809,7 +5809,7 @@
         <v>466</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18" hidden="1">
       <c r="A84" s="8" t="s">
         <v>65</v>
       </c>
@@ -5849,7 +5849,7 @@
         <v>469</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18" hidden="1">
       <c r="A85" s="8" t="s">
         <v>65</v>
       </c>
@@ -5887,7 +5887,7 @@
         <v>472</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18" hidden="1">
       <c r="A86" s="8" t="s">
         <v>65</v>
       </c>
@@ -5929,7 +5929,7 @@
         <v>474</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18" hidden="1">
       <c r="A87" s="8" t="s">
         <v>65</v>
       </c>
@@ -5969,7 +5969,7 @@
         <v>477</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18" hidden="1">
       <c r="A88" s="8" t="s">
         <v>65</v>
       </c>
@@ -6009,7 +6009,7 @@
         <v>480</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18" hidden="1">
       <c r="A89" s="8" t="s">
         <v>65</v>
       </c>
@@ -6047,7 +6047,7 @@
         <v>483</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18" hidden="1">
       <c r="A90" s="8" t="s">
         <v>65</v>
       </c>
@@ -6085,7 +6085,7 @@
         <v>486</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18" hidden="1">
       <c r="A91" s="6" t="s">
         <v>160</v>
       </c>
@@ -6125,7 +6125,7 @@
         <v>487</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18" hidden="1">
       <c r="A92" s="6" t="s">
         <v>160</v>
       </c>
@@ -6163,7 +6163,7 @@
         <v>489</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18" hidden="1">
       <c r="A93" s="8" t="s">
         <v>100</v>
       </c>
@@ -6201,7 +6201,7 @@
         <v>492</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18" hidden="1">
       <c r="A94" s="8" t="s">
         <v>100</v>
       </c>
@@ -6239,7 +6239,7 @@
         <v>494</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18" hidden="1">
       <c r="A95" s="6" t="s">
         <v>68</v>
       </c>
@@ -6281,7 +6281,7 @@
         <v>497</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18" hidden="1">
       <c r="A96" s="6" t="s">
         <v>68</v>
       </c>
@@ -6323,7 +6323,7 @@
         <v>499</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18" hidden="1">
       <c r="A97" s="6" t="s">
         <v>68</v>
       </c>
@@ -6365,7 +6365,7 @@
         <v>501</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18" hidden="1">
       <c r="A98" s="8" t="s">
         <v>62</v>
       </c>
@@ -6407,7 +6407,7 @@
         <v>503</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18" hidden="1">
       <c r="A99" s="8" t="s">
         <v>62</v>
       </c>
@@ -6449,7 +6449,7 @@
         <v>505</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18" hidden="1">
       <c r="A100" s="8" t="s">
         <v>62</v>
       </c>
@@ -6489,7 +6489,7 @@
         <v>507</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18" hidden="1">
       <c r="A101" s="6" t="s">
         <v>170</v>
       </c>
@@ -6527,7 +6527,7 @@
         <v>508</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18" hidden="1">
       <c r="A102" s="8" t="s">
         <v>175</v>
       </c>
@@ -6565,7 +6565,7 @@
         <v>511</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18" hidden="1">
       <c r="A103" s="8" t="s">
         <v>175</v>
       </c>
@@ -6603,7 +6603,7 @@
         <v>514</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18" hidden="1">
       <c r="A104" s="8" t="s">
         <v>175</v>
       </c>
@@ -6641,7 +6641,7 @@
         <v>517</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18" hidden="1">
       <c r="A105" s="8" t="s">
         <v>175</v>
       </c>
@@ -6679,7 +6679,7 @@
         <v>520</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18" hidden="1">
       <c r="A106" s="8" t="s">
         <v>175</v>
       </c>
@@ -6717,7 +6717,7 @@
         <v>523</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18" hidden="1">
       <c r="A107" s="8" t="s">
         <v>175</v>
       </c>
@@ -6755,7 +6755,7 @@
         <v>526</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18" hidden="1">
       <c r="A108" s="8" t="s">
         <v>175</v>
       </c>
@@ -6787,7 +6787,7 @@
         <v>529</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18" hidden="1">
       <c r="A109" s="8" t="s">
         <v>175</v>
       </c>
@@ -6819,7 +6819,7 @@
         <v>532</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18" hidden="1">
       <c r="A110" s="8" t="s">
         <v>175</v>
       </c>
@@ -6851,7 +6851,7 @@
         <v>536</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18" hidden="1">
       <c r="A111" s="8" t="s">
         <v>175</v>
       </c>
@@ -6883,7 +6883,7 @@
         <v>539</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18" hidden="1">
       <c r="A112" s="6" t="s">
         <v>178</v>
       </c>
@@ -6921,7 +6921,7 @@
         <v>542</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18" hidden="1">
       <c r="A113" s="6" t="s">
         <v>178</v>
       </c>
@@ -6959,7 +6959,7 @@
         <v>544</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18" hidden="1">
       <c r="A114" s="8" t="s">
         <v>96</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>547</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18" hidden="1">
       <c r="A115" s="8" t="s">
         <v>96</v>
       </c>
@@ -7035,7 +7035,7 @@
         <v>550</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18" hidden="1">
       <c r="A116" s="8" t="s">
         <v>96</v>
       </c>
@@ -7073,7 +7073,7 @@
         <v>553</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18" hidden="1">
       <c r="A117" s="8" t="s">
         <v>96</v>
       </c>
@@ -7111,7 +7111,7 @@
         <v>556</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18" hidden="1">
       <c r="A118" s="8" t="s">
         <v>96</v>
       </c>
@@ -7149,7 +7149,7 @@
         <v>559</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18" hidden="1">
       <c r="A119" s="8" t="s">
         <v>96</v>
       </c>
@@ -7187,7 +7187,7 @@
         <v>562</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18" hidden="1">
       <c r="A120" s="8" t="s">
         <v>96</v>
       </c>
@@ -7225,7 +7225,7 @@
         <v>565</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18" hidden="1">
       <c r="A121" s="8" t="s">
         <v>96</v>
       </c>
@@ -7263,7 +7263,7 @@
         <v>568</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18" hidden="1">
       <c r="A122" s="8" t="s">
         <v>96</v>
       </c>
@@ -7301,7 +7301,7 @@
         <v>571</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18" hidden="1">
       <c r="A123" s="8" t="s">
         <v>96</v>
       </c>
@@ -7339,7 +7339,7 @@
         <v>574</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18" hidden="1">
       <c r="A124" s="8" t="s">
         <v>96</v>
       </c>
@@ -7377,7 +7377,7 @@
         <v>577</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18" hidden="1">
       <c r="A125" s="8" t="s">
         <v>96</v>
       </c>
@@ -7415,7 +7415,7 @@
         <v>580</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18" hidden="1">
       <c r="A126" s="6" t="s">
         <v>57</v>
       </c>
@@ -7455,7 +7455,7 @@
         <v>583</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18" hidden="1">
       <c r="A127" s="6" t="s">
         <v>57</v>
       </c>
@@ -7493,7 +7493,7 @@
         <v>586</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18" hidden="1">
       <c r="A128" s="6" t="s">
         <v>57</v>
       </c>
@@ -7531,7 +7531,7 @@
         <v>589</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18" hidden="1">
       <c r="A129" s="6" t="s">
         <v>57</v>
       </c>
@@ -7569,7 +7569,7 @@
         <v>592</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18" hidden="1">
       <c r="A130" s="8" t="s">
         <v>184</v>
       </c>
@@ -7609,7 +7609,7 @@
         <v>595</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18" hidden="1">
       <c r="A131" s="8" t="s">
         <v>184</v>
       </c>
@@ -7649,7 +7649,7 @@
         <v>599</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18" hidden="1">
       <c r="A132" s="8" t="s">
         <v>184</v>
       </c>
@@ -7719,7 +7719,7 @@
         <v>604</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18" hidden="1">
       <c r="A134" s="8" t="s">
         <v>76</v>
       </c>
@@ -7761,7 +7761,7 @@
         <v>606</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18" hidden="1">
       <c r="A135" s="8" t="s">
         <v>76</v>
       </c>
@@ -7801,7 +7801,7 @@
         <v>610</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18" hidden="1">
       <c r="A136" s="8" t="s">
         <v>76</v>
       </c>
@@ -7841,7 +7841,7 @@
         <v>614</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18" hidden="1">
       <c r="A137" s="8" t="s">
         <v>76</v>
       </c>
@@ -7883,7 +7883,7 @@
         <v>618</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18" hidden="1">
       <c r="A138" s="8" t="s">
         <v>76</v>
       </c>
@@ -7923,7 +7923,7 @@
         <v>622</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18" hidden="1">
       <c r="A139" s="8" t="s">
         <v>76</v>
       </c>
@@ -7965,7 +7965,7 @@
         <v>626</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18" hidden="1">
       <c r="A140" s="8" t="s">
         <v>76</v>
       </c>
@@ -7999,7 +7999,7 @@
         <v>629</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18" hidden="1">
       <c r="A141" s="6" t="s">
         <v>80</v>
       </c>
@@ -8041,7 +8041,7 @@
         <v>632</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18" hidden="1">
       <c r="A142" s="8" t="s">
         <v>195</v>
       </c>
@@ -8079,7 +8079,7 @@
         <v>636</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18" hidden="1">
       <c r="A143" s="6" t="s">
         <v>199</v>
       </c>

</xml_diff>

<commit_message>
adding CDM views to the view model
</commit_message>
<xml_diff>
--- a/cfihos_src/cdm_export.xlsx
+++ b/cfihos_src/cdm_export.xlsx
@@ -2575,7 +2575,7 @@
     <col min="16" max="16" style="10" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="4" t="s">
         <v>203</v>
       </c>
@@ -2595,7 +2595,7 @@
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
       <c r="A2" s="5" t="s">
         <v>104</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
       <c r="A3" s="6" t="s">
         <v>82</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>218</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
       <c r="A4" s="6" t="s">
         <v>82</v>
       </c>
@@ -2729,7 +2729,7 @@
         <v>223</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
       <c r="A5" s="6" t="s">
         <v>82</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>228</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
       <c r="A6" s="6" t="s">
         <v>82</v>
       </c>
@@ -2811,7 +2811,7 @@
         <v>233</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
       <c r="A7" s="6" t="s">
         <v>82</v>
       </c>
@@ -2853,7 +2853,7 @@
         <v>236</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
       <c r="A8" s="6" t="s">
         <v>82</v>
       </c>
@@ -2895,7 +2895,7 @@
         <v>239</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
       <c r="A9" s="6" t="s">
         <v>82</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>244</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
       <c r="A10" s="6" t="s">
         <v>82</v>
       </c>
@@ -2963,7 +2963,7 @@
         <v>249</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
       <c r="A11" s="6" t="s">
         <v>82</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>253</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
       <c r="A12" s="6" t="s">
         <v>82</v>
       </c>
@@ -3031,7 +3031,7 @@
         <v>257</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
       <c r="A13" s="6" t="s">
         <v>82</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>260</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
       <c r="A14" s="8" t="s">
         <v>85</v>
       </c>
@@ -3105,7 +3105,7 @@
         <v>263</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18">
       <c r="A15" s="8" t="s">
         <v>85</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>266</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18">
       <c r="A16" s="8" t="s">
         <v>85</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>269</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18">
       <c r="A17" s="8" t="s">
         <v>85</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>272</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
       <c r="A18" s="6" t="s">
         <v>115</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>275</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
       <c r="A19" s="6" t="s">
         <v>115</v>
       </c>
@@ -3305,7 +3305,7 @@
         <v>278</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
       <c r="A20" s="6" t="s">
         <v>115</v>
       </c>
@@ -3383,7 +3383,7 @@
         <v>284</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18">
       <c r="A22" s="6" t="s">
         <v>115</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>288</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18">
       <c r="A23" s="6" t="s">
         <v>115</v>
       </c>
@@ -3459,7 +3459,7 @@
         <v>291</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18">
       <c r="A24" s="6" t="s">
         <v>115</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>294</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18">
       <c r="A25" s="8" t="s">
         <v>118</v>
       </c>
@@ -3537,7 +3537,7 @@
         <v>296</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18">
       <c r="A26" s="8" t="s">
         <v>118</v>
       </c>
@@ -3575,7 +3575,7 @@
         <v>299</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18">
       <c r="A27" s="6" t="s">
         <v>59</v>
       </c>
@@ -3613,7 +3613,7 @@
         <v>302</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18">
       <c r="A28" s="6" t="s">
         <v>59</v>
       </c>
@@ -3651,7 +3651,7 @@
         <v>306</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18">
       <c r="A29" s="8" t="s">
         <v>124</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>309</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="8" t="s">
         <v>124</v>
       </c>
@@ -3727,7 +3727,7 @@
         <v>312</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="8" t="s">
         <v>124</v>
       </c>
@@ -3765,7 +3765,7 @@
         <v>315</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="8" t="s">
         <v>124</v>
       </c>
@@ -3803,7 +3803,7 @@
         <v>318</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="8" t="s">
         <v>124</v>
       </c>
@@ -3841,7 +3841,7 @@
         <v>321</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18">
       <c r="A34" s="8" t="s">
         <v>124</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>324</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18">
       <c r="A35" s="8" t="s">
         <v>124</v>
       </c>
@@ -3917,7 +3917,7 @@
         <v>327</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18">
       <c r="A36" s="8" t="s">
         <v>124</v>
       </c>
@@ -3955,7 +3955,7 @@
         <v>330</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18">
       <c r="A37" s="8" t="s">
         <v>124</v>
       </c>
@@ -3993,7 +3993,7 @@
         <v>333</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18">
       <c r="A38" s="6" t="s">
         <v>90</v>
       </c>
@@ -4035,7 +4035,7 @@
         <v>337</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18">
       <c r="A39" s="6" t="s">
         <v>90</v>
       </c>
@@ -4077,7 +4077,7 @@
         <v>339</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18">
       <c r="A40" s="6" t="s">
         <v>90</v>
       </c>
@@ -4119,7 +4119,7 @@
         <v>341</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18">
       <c r="A41" s="8" t="s">
         <v>130</v>
       </c>
@@ -4159,7 +4159,7 @@
         <v>342</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18">
       <c r="A42" s="8" t="s">
         <v>130</v>
       </c>
@@ -4199,7 +4199,7 @@
         <v>344</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18">
       <c r="A43" s="8" t="s">
         <v>130</v>
       </c>
@@ -4277,7 +4277,7 @@
         <v>349</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18">
       <c r="A45" s="8" t="s">
         <v>130</v>
       </c>
@@ -4315,7 +4315,7 @@
         <v>352</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18">
       <c r="A46" s="8" t="s">
         <v>130</v>
       </c>
@@ -4353,7 +4353,7 @@
         <v>355</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18">
       <c r="A47" s="6" t="s">
         <v>98</v>
       </c>
@@ -4395,7 +4395,7 @@
         <v>358</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18">
       <c r="A48" s="6" t="s">
         <v>98</v>
       </c>
@@ -4437,7 +4437,7 @@
         <v>362</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18">
       <c r="A49" s="6" t="s">
         <v>98</v>
       </c>
@@ -4479,7 +4479,7 @@
         <v>366</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18">
       <c r="A50" s="6" t="s">
         <v>98</v>
       </c>
@@ -4521,7 +4521,7 @@
         <v>369</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18">
       <c r="A51" s="6" t="s">
         <v>98</v>
       </c>
@@ -4563,7 +4563,7 @@
         <v>371</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18">
       <c r="A52" s="6" t="s">
         <v>98</v>
       </c>
@@ -4597,7 +4597,7 @@
         <v>374</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18">
       <c r="A53" s="6" t="s">
         <v>98</v>
       </c>
@@ -4631,7 +4631,7 @@
         <v>376</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18">
       <c r="A54" s="8" t="s">
         <v>93</v>
       </c>
@@ -4669,7 +4669,7 @@
         <v>379</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="8" t="s">
         <v>93</v>
       </c>
@@ -4707,7 +4707,7 @@
         <v>382</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18">
       <c r="A56" s="8" t="s">
         <v>93</v>
       </c>
@@ -4745,7 +4745,7 @@
         <v>385</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18">
       <c r="A57" s="8" t="s">
         <v>93</v>
       </c>
@@ -4783,7 +4783,7 @@
         <v>388</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18">
       <c r="A58" s="6" t="s">
         <v>55</v>
       </c>
@@ -4825,7 +4825,7 @@
         <v>393</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18">
       <c r="A59" s="6" t="s">
         <v>55</v>
       </c>
@@ -4867,7 +4867,7 @@
         <v>397</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18">
       <c r="A60" s="8" t="s">
         <v>71</v>
       </c>
@@ -4909,7 +4909,7 @@
         <v>399</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18">
       <c r="A61" s="8" t="s">
         <v>71</v>
       </c>
@@ -4949,7 +4949,7 @@
         <v>403</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18">
       <c r="A62" s="8" t="s">
         <v>71</v>
       </c>
@@ -4991,7 +4991,7 @@
         <v>405</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18">
       <c r="A63" s="8" t="s">
         <v>71</v>
       </c>
@@ -5031,7 +5031,7 @@
         <v>409</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18">
       <c r="A64" s="6" t="s">
         <v>143</v>
       </c>
@@ -5071,7 +5071,7 @@
         <v>412</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18">
       <c r="A65" s="6" t="s">
         <v>143</v>
       </c>
@@ -5109,7 +5109,7 @@
         <v>415</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18">
       <c r="A66" s="8" t="s">
         <v>120</v>
       </c>
@@ -5145,7 +5145,7 @@
         <v>417</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18">
       <c r="A67" s="8" t="s">
         <v>120</v>
       </c>
@@ -5181,7 +5181,7 @@
         <v>419</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18">
       <c r="A68" s="8" t="s">
         <v>120</v>
       </c>
@@ -5217,7 +5217,7 @@
         <v>421</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18">
       <c r="A69" s="8" t="s">
         <v>120</v>
       </c>
@@ -5255,7 +5255,7 @@
         <v>422</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18">
       <c r="A70" s="6" t="s">
         <v>148</v>
       </c>
@@ -5295,7 +5295,7 @@
         <v>425</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18">
       <c r="A71" s="6" t="s">
         <v>148</v>
       </c>
@@ -5335,7 +5335,7 @@
         <v>428</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18">
       <c r="A72" s="6" t="s">
         <v>148</v>
       </c>
@@ -5375,7 +5375,7 @@
         <v>431</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18">
       <c r="A73" s="6" t="s">
         <v>148</v>
       </c>
@@ -5415,7 +5415,7 @@
         <v>434</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18">
       <c r="A74" s="6" t="s">
         <v>148</v>
       </c>
@@ -5455,7 +5455,7 @@
         <v>437</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18">
       <c r="A75" s="6" t="s">
         <v>148</v>
       </c>
@@ -5527,7 +5527,7 @@
         <v>443</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18">
       <c r="A77" s="6" t="s">
         <v>88</v>
       </c>
@@ -5569,7 +5569,7 @@
         <v>447</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18">
       <c r="A78" s="6" t="s">
         <v>88</v>
       </c>
@@ -5609,7 +5609,7 @@
         <v>451</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18">
       <c r="A79" s="6" t="s">
         <v>88</v>
       </c>
@@ -5649,7 +5649,7 @@
         <v>455</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18">
       <c r="A80" s="6" t="s">
         <v>88</v>
       </c>
@@ -5691,7 +5691,7 @@
         <v>459</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18">
       <c r="A81" s="6" t="s">
         <v>88</v>
       </c>
@@ -5733,7 +5733,7 @@
         <v>461</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18">
       <c r="A82" s="6" t="s">
         <v>88</v>
       </c>
@@ -5775,7 +5775,7 @@
         <v>463</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18">
       <c r="A83" s="6" t="s">
         <v>88</v>
       </c>
@@ -5809,7 +5809,7 @@
         <v>466</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18">
       <c r="A84" s="8" t="s">
         <v>65</v>
       </c>
@@ -5849,7 +5849,7 @@
         <v>469</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18">
       <c r="A85" s="8" t="s">
         <v>65</v>
       </c>
@@ -5887,7 +5887,7 @@
         <v>472</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18">
       <c r="A86" s="8" t="s">
         <v>65</v>
       </c>
@@ -5929,7 +5929,7 @@
         <v>474</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18">
       <c r="A87" s="8" t="s">
         <v>65</v>
       </c>
@@ -5969,7 +5969,7 @@
         <v>477</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18">
       <c r="A88" s="8" t="s">
         <v>65</v>
       </c>
@@ -6009,7 +6009,7 @@
         <v>480</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18">
       <c r="A89" s="8" t="s">
         <v>65</v>
       </c>
@@ -6047,7 +6047,7 @@
         <v>483</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18">
       <c r="A90" s="8" t="s">
         <v>65</v>
       </c>
@@ -6085,7 +6085,7 @@
         <v>486</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18">
       <c r="A91" s="6" t="s">
         <v>160</v>
       </c>
@@ -6125,7 +6125,7 @@
         <v>487</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18">
       <c r="A92" s="6" t="s">
         <v>160</v>
       </c>
@@ -6163,7 +6163,7 @@
         <v>489</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18">
       <c r="A93" s="8" t="s">
         <v>100</v>
       </c>
@@ -6201,7 +6201,7 @@
         <v>492</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18">
       <c r="A94" s="8" t="s">
         <v>100</v>
       </c>
@@ -6239,7 +6239,7 @@
         <v>494</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18">
       <c r="A95" s="6" t="s">
         <v>68</v>
       </c>
@@ -6281,7 +6281,7 @@
         <v>497</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18">
       <c r="A96" s="6" t="s">
         <v>68</v>
       </c>
@@ -6323,7 +6323,7 @@
         <v>499</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18">
       <c r="A97" s="6" t="s">
         <v>68</v>
       </c>
@@ -6365,7 +6365,7 @@
         <v>501</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18">
       <c r="A98" s="8" t="s">
         <v>62</v>
       </c>
@@ -6407,7 +6407,7 @@
         <v>503</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18">
       <c r="A99" s="8" t="s">
         <v>62</v>
       </c>
@@ -6449,7 +6449,7 @@
         <v>505</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18">
       <c r="A100" s="8" t="s">
         <v>62</v>
       </c>
@@ -6489,7 +6489,7 @@
         <v>507</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18">
       <c r="A101" s="6" t="s">
         <v>170</v>
       </c>
@@ -6527,7 +6527,7 @@
         <v>508</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18">
       <c r="A102" s="8" t="s">
         <v>175</v>
       </c>
@@ -6565,7 +6565,7 @@
         <v>511</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18">
       <c r="A103" s="8" t="s">
         <v>175</v>
       </c>
@@ -6603,7 +6603,7 @@
         <v>514</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18">
       <c r="A104" s="8" t="s">
         <v>175</v>
       </c>
@@ -6641,7 +6641,7 @@
         <v>517</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18">
       <c r="A105" s="8" t="s">
         <v>175</v>
       </c>
@@ -6679,7 +6679,7 @@
         <v>520</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18">
       <c r="A106" s="8" t="s">
         <v>175</v>
       </c>
@@ -6717,7 +6717,7 @@
         <v>523</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18">
       <c r="A107" s="8" t="s">
         <v>175</v>
       </c>
@@ -6755,7 +6755,7 @@
         <v>526</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18">
       <c r="A108" s="8" t="s">
         <v>175</v>
       </c>
@@ -6787,7 +6787,7 @@
         <v>529</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18">
       <c r="A109" s="8" t="s">
         <v>175</v>
       </c>
@@ -6819,7 +6819,7 @@
         <v>532</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
       <c r="A110" s="8" t="s">
         <v>175</v>
       </c>
@@ -6851,7 +6851,7 @@
         <v>536</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
       <c r="A111" s="8" t="s">
         <v>175</v>
       </c>
@@ -6883,7 +6883,7 @@
         <v>539</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
       <c r="A112" s="6" t="s">
         <v>178</v>
       </c>
@@ -6921,7 +6921,7 @@
         <v>542</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
       <c r="A113" s="6" t="s">
         <v>178</v>
       </c>
@@ -6959,7 +6959,7 @@
         <v>544</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
       <c r="A114" s="8" t="s">
         <v>96</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>547</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
       <c r="A115" s="8" t="s">
         <v>96</v>
       </c>
@@ -7035,7 +7035,7 @@
         <v>550</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
       <c r="A116" s="8" t="s">
         <v>96</v>
       </c>
@@ -7073,7 +7073,7 @@
         <v>553</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
       <c r="A117" s="8" t="s">
         <v>96</v>
       </c>
@@ -7111,7 +7111,7 @@
         <v>556</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
       <c r="A118" s="8" t="s">
         <v>96</v>
       </c>
@@ -7149,7 +7149,7 @@
         <v>559</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
       <c r="A119" s="8" t="s">
         <v>96</v>
       </c>
@@ -7187,7 +7187,7 @@
         <v>562</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
       <c r="A120" s="8" t="s">
         <v>96</v>
       </c>
@@ -7225,7 +7225,7 @@
         <v>565</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
       <c r="A121" s="8" t="s">
         <v>96</v>
       </c>
@@ -7263,7 +7263,7 @@
         <v>568</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
       <c r="A122" s="8" t="s">
         <v>96</v>
       </c>
@@ -7301,7 +7301,7 @@
         <v>571</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
       <c r="A123" s="8" t="s">
         <v>96</v>
       </c>
@@ -7339,7 +7339,7 @@
         <v>574</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
       <c r="A124" s="8" t="s">
         <v>96</v>
       </c>
@@ -7377,7 +7377,7 @@
         <v>577</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
       <c r="A125" s="8" t="s">
         <v>96</v>
       </c>
@@ -7415,7 +7415,7 @@
         <v>580</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
       <c r="A126" s="6" t="s">
         <v>57</v>
       </c>
@@ -7455,7 +7455,7 @@
         <v>583</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
       <c r="A127" s="6" t="s">
         <v>57</v>
       </c>
@@ -7493,7 +7493,7 @@
         <v>586</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
       <c r="A128" s="6" t="s">
         <v>57</v>
       </c>
@@ -7531,7 +7531,7 @@
         <v>589</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
       <c r="A129" s="6" t="s">
         <v>57</v>
       </c>
@@ -7569,7 +7569,7 @@
         <v>592</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
       <c r="A130" s="8" t="s">
         <v>184</v>
       </c>
@@ -7609,7 +7609,7 @@
         <v>595</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
       <c r="A131" s="8" t="s">
         <v>184</v>
       </c>
@@ -7649,7 +7649,7 @@
         <v>599</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
       <c r="A132" s="8" t="s">
         <v>184</v>
       </c>
@@ -7719,7 +7719,7 @@
         <v>604</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
       <c r="A134" s="8" t="s">
         <v>76</v>
       </c>
@@ -7761,7 +7761,7 @@
         <v>606</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
       <c r="A135" s="8" t="s">
         <v>76</v>
       </c>
@@ -7801,7 +7801,7 @@
         <v>610</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
       <c r="A136" s="8" t="s">
         <v>76</v>
       </c>
@@ -7841,7 +7841,7 @@
         <v>614</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
       <c r="A137" s="8" t="s">
         <v>76</v>
       </c>
@@ -7883,7 +7883,7 @@
         <v>618</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
       <c r="A138" s="8" t="s">
         <v>76</v>
       </c>
@@ -7923,7 +7923,7 @@
         <v>622</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
       <c r="A139" s="8" t="s">
         <v>76</v>
       </c>
@@ -7965,7 +7965,7 @@
         <v>626</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
       <c r="A140" s="8" t="s">
         <v>76</v>
       </c>
@@ -7999,7 +7999,7 @@
         <v>629</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
       <c r="A141" s="6" t="s">
         <v>80</v>
       </c>
@@ -8041,7 +8041,7 @@
         <v>632</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
       <c r="A142" s="8" t="s">
         <v>195</v>
       </c>
@@ -8079,7 +8079,7 @@
         <v>636</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18" hidden="1">
+    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="19.5">
       <c r="A143" s="6" t="s">
         <v>199</v>
       </c>

</xml_diff>